<commit_message>
Improved Credits tab on dashboard
</commit_message>
<xml_diff>
--- a/האגמית7_כספים_2026.xlsx
+++ b/האגמית7_כספים_2026.xlsx
@@ -7448,10 +7448,10 @@
         <v>0</v>
       </c>
       <c r="C9" s="246" t="n">
-        <v>48.38</v>
+        <v>0</v>
       </c>
       <c r="D9" s="246" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="E9" s="246" t="n">
         <v>77</v>

</xml_diff>

<commit_message>
dashboard credit improvements, inc 500 petty cash
</commit_message>
<xml_diff>
--- a/האגמית7_כספים_2026.xlsx
+++ b/האגמית7_כספים_2026.xlsx
@@ -3478,7 +3478,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>250</v>
+        <v>500</v>
       </c>
       <c r="S2" s="62" t="n"/>
       <c r="X2">
@@ -3510,10 +3510,10 @@
         <v>350</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -3534,6 +3534,9 @@
         <v>0</v>
       </c>
       <c r="P3" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
         <v>0</v>
       </c>
       <c r="X3">
@@ -3644,6 +3647,9 @@
       <c r="P5" s="63" t="n">
         <v>0</v>
       </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
       <c r="S5" s="62" t="n"/>
       <c r="X5">
         <f t="array" ref="X5">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B5, _xlpm.payments, E5:P5, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
@@ -3873,6 +3879,9 @@
       <c r="P9" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
       <c r="X9">
         <f t="array" ref="X9">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B9, _xlpm.payments, E9:P9, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -3925,6 +3934,9 @@
         <v>0</v>
       </c>
       <c r="P10" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
         <v>0</v>
       </c>
       <c r="S10" s="62" t="n"/>
@@ -3979,6 +3991,9 @@
       <c r="P11" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
       <c r="S11" t="n">
         <v>4590840</v>
       </c>
@@ -4144,6 +4159,9 @@
       <c r="P14" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
       <c r="X14">
         <f t="array" ref="X14">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B14, _xlpm.payments, E14:P14, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -4176,10 +4194,10 @@
         <v>350</v>
       </c>
       <c r="H15" s="62" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="I15" s="62" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="J15" s="62" t="n">
         <v>0</v>
@@ -4200,6 +4218,9 @@
         <v>0</v>
       </c>
       <c r="P15" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="S15" s="62" t="n"/>
@@ -4442,18 +4463,42 @@
         </is>
       </c>
       <c r="D20" s="62" t="n"/>
-      <c r="E20" s="169" t="n"/>
-      <c r="F20" s="66" t="n"/>
-      <c r="G20" s="66" t="n"/>
-      <c r="H20" s="66" t="n"/>
-      <c r="I20" s="66" t="n"/>
-      <c r="J20" s="66" t="n"/>
-      <c r="K20" s="66" t="n"/>
-      <c r="L20" s="66" t="n"/>
-      <c r="M20" s="66" t="n"/>
-      <c r="N20" s="66" t="n"/>
-      <c r="O20" s="66" t="n"/>
-      <c r="P20" s="67" t="n"/>
+      <c r="E20" s="169" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="66" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="67" t="n">
+        <v>0</v>
+      </c>
       <c r="Q20" t="n">
         <v>350</v>
       </c>
@@ -4509,6 +4554,9 @@
       <c r="P21" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
       <c r="X21">
         <f t="array" ref="X21">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B21, _xlpm.payments, E21:P21, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -4614,6 +4662,9 @@
       <c r="P23" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q23" t="n">
+        <v>200</v>
+      </c>
       <c r="X23">
         <f t="array" ref="X23">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B23, _xlpm.payments, E23:P23, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -4800,18 +4851,42 @@
           <t>שוורץ</t>
         </is>
       </c>
-      <c r="E27" s="170" t="n"/>
-      <c r="F27" s="48" t="n"/>
-      <c r="G27" s="48" t="n"/>
-      <c r="H27" s="48" t="n"/>
-      <c r="I27" s="48" t="n"/>
-      <c r="J27" s="48" t="n"/>
-      <c r="K27" s="48" t="n"/>
-      <c r="L27" s="48" t="n"/>
-      <c r="M27" s="48" t="n"/>
-      <c r="N27" s="48" t="n"/>
-      <c r="O27" s="48" t="n"/>
-      <c r="P27" s="49" t="n"/>
+      <c r="E27" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="49" t="n">
+        <v>0</v>
+      </c>
       <c r="Q27" t="n">
         <v>500</v>
       </c>
@@ -5042,6 +5117,9 @@
       <c r="P31" s="156" t="n">
         <v>0</v>
       </c>
+      <c r="Q31" t="n">
+        <v>500</v>
+      </c>
       <c r="X31">
         <f t="array" ref="X31">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B31, _xlpm.payments, E31:P31, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -5173,18 +5251,42 @@
           <t>וילצר</t>
         </is>
       </c>
-      <c r="E34" s="170" t="n"/>
-      <c r="F34" s="48" t="n"/>
-      <c r="G34" s="48" t="n"/>
-      <c r="H34" s="48" t="n"/>
-      <c r="I34" s="48" t="n"/>
-      <c r="J34" s="48" t="n"/>
-      <c r="K34" s="48" t="n"/>
-      <c r="L34" s="48" t="n"/>
-      <c r="M34" s="48" t="n"/>
-      <c r="N34" s="48" t="n"/>
-      <c r="O34" s="48" t="n"/>
-      <c r="P34" s="49" t="n"/>
+      <c r="E34" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="49" t="n">
+        <v>0</v>
+      </c>
       <c r="Q34" t="n">
         <v>500</v>
       </c>
@@ -5354,6 +5456,9 @@
       <c r="P37" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
       <c r="X37">
         <f t="array" ref="X37">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B37, _xlpm.payments, E37:P37, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -5410,6 +5515,9 @@
       <c r="P38" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q38" t="n">
+        <v>0</v>
+      </c>
       <c r="X38">
         <f t="array" ref="X38">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B38, _xlpm.payments, E38:P38, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -5425,18 +5533,45 @@
           <t>ברכה</t>
         </is>
       </c>
-      <c r="E39" s="170" t="n"/>
-      <c r="F39" s="48" t="n"/>
-      <c r="G39" s="48" t="n"/>
-      <c r="H39" s="48" t="n"/>
-      <c r="I39" s="48" t="n"/>
-      <c r="J39" s="48" t="n"/>
-      <c r="K39" s="48" t="n"/>
-      <c r="L39" s="48" t="n"/>
-      <c r="M39" s="48" t="n"/>
-      <c r="N39" s="48" t="n"/>
-      <c r="O39" s="48" t="n"/>
-      <c r="P39" s="49" t="n"/>
+      <c r="E39" s="170" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O39" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
       <c r="X39">
         <f t="array" ref="X39">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B39, _xlpm.payments, E39:P39, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -5602,6 +5737,9 @@
       <c r="P42" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
       <c r="X42">
         <f t="array" ref="X42">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B42, _xlpm.payments, E42:P42, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -5653,6 +5791,9 @@
       <c r="P43" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q43" t="n">
+        <v>0</v>
+      </c>
       <c r="X43">
         <f t="array" ref="X43">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B43, _xlpm.payments, E43:P43, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -6056,6 +6197,9 @@
       <c r="P50" s="63" t="n">
         <v>0</v>
       </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
       <c r="R50" t="inlineStr">
         <is>
           <t>הו"ק ב29 לכל חודש</t>
@@ -6115,6 +6259,9 @@
       <c r="P51" s="156" t="n">
         <v>0</v>
       </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
       <c r="R51" t="inlineStr">
         <is>
           <t>חוב נוב + דצ +ינו 30X3 שקל</t>
@@ -6179,6 +6326,9 @@
       <c r="P52" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q52" t="n">
+        <v>0</v>
+      </c>
       <c r="S52" t="n">
         <v>4691410</v>
       </c>
@@ -6288,6 +6438,9 @@
       <c r="P54" s="172" t="n">
         <v>0</v>
       </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
       <c r="R54" t="inlineStr">
         <is>
           <t>הו"ק ב28 לכל חודש</t>
@@ -6347,6 +6500,9 @@
       <c r="P55" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
       <c r="S55" t="n">
         <v>4763312</v>
       </c>
@@ -6522,6 +6678,9 @@
       <c r="P58" s="46" t="n">
         <v>0</v>
       </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
       <c r="X58">
         <f t="array" ref="X58">_xlfn.LET(_xlpm.exclude_list, {19,26,33,38}, _xlpm.current_month_idx, MONTH(TODAY()), _xlpm.month_names, {"ינואר","פברואר","מרץ","אפריל","מאי","יוני","יולי","אוגוסט","ספטמבר","אוקטובר","נובמבר","דצמבר"}, _xlpm.target, 350, _xlpm.apartment, B58, _xlpm.payments, E58:P58, IF(ISNUMBER(MATCH(_xlpm.apartment, _xlpm.exclude_list, 0)), "", _xlfn.LET(_xlpm.debt_list, _xlfn.MAP(_xlfn.SEQUENCE(1, 12), _xlpm.month_names, _xlpm.payments, _xlfn.LAMBDA(_xlpm.idx,_xlpm.m_name,_xlpm.p_val, IF(_xlpm.idx &gt; _xlpm.current_month_idx, "", IF(OR(ISBLANK(_xlpm.p_val), _xlpm.p_val = ""), _xlpm.m_name &amp; " (חוב " &amp; _xlpm.target &amp; ")", IF(_xlpm.p_val &lt; _xlpm.target, _xlpm.m_name &amp; " (חוב " &amp; (_xlpm.target - _xlpm.p_val) &amp; ")", ""))))), _xlpm.summary, _xlfn.TEXTJOIN(", ", TRUE, _xlpm.debt_list), IF(_xlpm.summary &lt;&gt; "", "דירה " &amp; _xlpm.apartment &amp; " - " &amp; _xlpm.summary, ""))))</f>
         <v/>
@@ -6547,7 +6706,7 @@
         <v>350</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
@@ -6571,6 +6730,9 @@
         <v>0</v>
       </c>
       <c r="P59" s="156" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
         <v>0</v>
       </c>
       <c r="S59" t="n">
@@ -6628,6 +6790,9 @@
         <v>0</v>
       </c>
       <c r="P60" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" t="n">
         <v>0</v>
       </c>
       <c r="S60" s="61" t="inlineStr">
@@ -6984,7 +7149,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24.7109375" bestFit="1" customWidth="1" style="177" min="1" max="1"/>
@@ -7199,7 +7364,7 @@
         <v>3233.77</v>
       </c>
       <c r="E4" s="246" t="n">
-        <v>0</v>
+        <v>3353.66</v>
       </c>
       <c r="F4" s="246" t="n">
         <v>0</v>
@@ -7403,7 +7568,7 @@
         <v>90.77</v>
       </c>
       <c r="E8" s="246" t="n">
-        <v>0</v>
+        <v>90.77</v>
       </c>
       <c r="F8" s="246" t="n">
         <v>0</v>
@@ -8004,8 +8169,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23" ht="57.75" customHeight="1" s="177">
       <c r="A23" t="inlineStr">
         <is>
@@ -8049,13 +8212,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="159" t="inlineStr">
         <is>
@@ -8107,24 +8263,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <conditionalFormatting sqref="B20:M20">
     <cfRule type="colorScale" priority="1">
@@ -20428,7 +20566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22109,6 +22247,105 @@
       <c r="F51" t="inlineStr">
         <is>
           <t>הפקדת שיק</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>700</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>הכנסה מדיירים</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>2</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>פיליפ אלברט 10-916-004497512 וועד בית אפריל ומאי דירה 2</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>העברה מאת: פיליפ אלברט 10-916-004497512 וועד בית אפריל ומאי דירה 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>350</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>הכנסה מדיירים</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>58</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>אליאס סמעאן 10-877-003268585 תשלום</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>העברה מאת: אליאס סמעאן 10-877-003268585 תשלום</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>27/04/2026</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>הכנסה מדיירים</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>14</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ירין חיים מל 10-882-046518869 ועד בית</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>העברה דיגיטל</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>העברה מאת: ירין חיים מל 10-882-046518869 ועד בית</t>
         </is>
       </c>
     </row>
@@ -22123,7 +22360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22443,6 +22680,56 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>24/04/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-90.77</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>פרטנר</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>חברת פרטנר</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>חברת פרטנר ת-י</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>26/04/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-3353.66</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>חשמל ציבורי</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>חברת החשמל</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>חברת החשמל ל-י</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>